<commit_message>
dimensional model and source to target mapping
</commit_message>
<xml_diff>
--- a/NorthWind WRK.xlsx
+++ b/NorthWind WRK.xlsx
@@ -8,18 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Analytics_Engineering\analytics-engineering-bootcamp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FDF39C-6097-4E50-8563-6A88C57B0E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34157A8-7A24-4FB2-9E2B-E881CCE1078B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="894" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="894" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BusMatrix-HighLevelEntites-Comp" sheetId="3" r:id="rId1"/>
     <sheet name="BusMatrix-Detailed-NorthWind-Co" sheetId="6" r:id="rId2"/>
-    <sheet name="source_to_target_mapping" sheetId="9" r:id="rId3"/>
-    <sheet name="source_to_target_mapping stagin" sheetId="12" r:id="rId4"/>
+    <sheet name="src_to_target_mapping data lake" sheetId="9" r:id="rId3"/>
+    <sheet name="src_to_target_map staging layer" sheetId="12" r:id="rId4"/>
     <sheet name="Dimensional Model " sheetId="15" r:id="rId5"/>
-    <sheet name="source_to_target_mapping wareho" sheetId="18" r:id="rId6"/>
-    <sheet name="source_to_target_mapping(OBT)" sheetId="21" r:id="rId7"/>
+    <sheet name="src_to_target_map warehouse" sheetId="18" r:id="rId6"/>
+    <sheet name="src_to_target_map (OBT)" sheetId="21" r:id="rId7"/>
     <sheet name="Orignial source_to_target_mappi" sheetId="22" state="hidden" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -873,7 +873,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -905,8 +905,22 @@
       <color rgb="FF707070"/>
       <name val="Roboto"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -973,6 +987,24 @@
         <bgColor rgb="FFF9CB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -995,7 +1027,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1072,13 +1104,31 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1483,7 +1533,9 @@
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
     <col min="6" max="10" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1684,20 +1736,20 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="12"/>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
       <c r="O1" s="13"/>
     </row>
     <row r="2" spans="1:15">
@@ -8276,23 +8328,23 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="12"/>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="39" t="s">
         <v>202</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="J1" s="34" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="J1" s="41" t="s">
         <v>203</v>
       </c>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
       <c r="P1" s="13"/>
     </row>
     <row r="2" spans="1:16">
@@ -9086,62 +9138,62 @@
       </c>
       <c r="O21" s="18"/>
     </row>
-    <row r="22" spans="1:32">
-      <c r="A22" s="18">
+    <row r="22" spans="1:32" s="34" customFormat="1">
+      <c r="A22" s="32">
         <v>19</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="18" t="s">
+      <c r="B22" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="32" t="s">
         <v>205</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="H22" s="18" t="str">
+      <c r="H22" s="32" t="str">
         <f t="shared" si="0"/>
         <v>insertion_timestamp,</v>
       </c>
-      <c r="J22" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K22" s="18" t="s">
+      <c r="J22" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="K22" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="L22" s="18" t="s">
+      <c r="L22" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="M22" s="18" t="s">
+      <c r="M22" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="N22" s="18" t="s">
+      <c r="N22" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="O22" s="20"/>
-      <c r="P22" s="20"/>
-      <c r="Q22" s="20"/>
-      <c r="R22" s="20"/>
-      <c r="S22" s="20"/>
-      <c r="T22" s="20"/>
-      <c r="U22" s="20"/>
-      <c r="V22" s="20"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="20"/>
-      <c r="Y22" s="20"/>
-      <c r="Z22" s="20"/>
-      <c r="AA22" s="20"/>
-      <c r="AB22" s="20"/>
-      <c r="AC22" s="20"/>
-      <c r="AD22" s="20"/>
-      <c r="AE22" s="20"/>
-      <c r="AF22" s="20"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="35"/>
+      <c r="R22" s="35"/>
+      <c r="S22" s="35"/>
+      <c r="T22" s="35"/>
+      <c r="U22" s="35"/>
+      <c r="V22" s="35"/>
+      <c r="W22" s="35"/>
+      <c r="X22" s="35"/>
+      <c r="Y22" s="35"/>
+      <c r="Z22" s="35"/>
+      <c r="AA22" s="35"/>
+      <c r="AB22" s="35"/>
+      <c r="AC22" s="35"/>
+      <c r="AD22" s="35"/>
+      <c r="AE22" s="35"/>
+      <c r="AF22" s="35"/>
     </row>
     <row r="23" spans="1:32">
       <c r="A23" s="16" t="s">
@@ -9812,59 +9864,59 @@
       </c>
       <c r="O41" s="18"/>
     </row>
-    <row r="42" spans="1:32">
-      <c r="A42" s="18">
+    <row r="42" spans="1:32" s="34" customFormat="1">
+      <c r="A42" s="32">
         <v>19</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="18" t="s">
+      <c r="B42" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F42" s="18" t="s">
+      <c r="F42" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G42" s="18"/>
-      <c r="J42" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K42" s="18" t="s">
+      <c r="G42" s="32"/>
+      <c r="J42" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="K42" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="L42" s="18" t="s">
+      <c r="L42" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="M42" s="18" t="s">
+      <c r="M42" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="N42" s="18" t="s">
+      <c r="N42" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="O42" s="20"/>
-      <c r="P42" s="20"/>
-      <c r="Q42" s="20"/>
-      <c r="R42" s="20"/>
-      <c r="S42" s="20"/>
-      <c r="T42" s="20"/>
-      <c r="U42" s="20"/>
-      <c r="V42" s="20"/>
-      <c r="W42" s="20"/>
-      <c r="X42" s="20"/>
-      <c r="Y42" s="20"/>
-      <c r="Z42" s="20"/>
-      <c r="AA42" s="20"/>
-      <c r="AB42" s="20"/>
-      <c r="AC42" s="20"/>
-      <c r="AD42" s="20"/>
-      <c r="AE42" s="20"/>
-      <c r="AF42" s="20"/>
+      <c r="O42" s="35"/>
+      <c r="P42" s="35"/>
+      <c r="Q42" s="35"/>
+      <c r="R42" s="35"/>
+      <c r="S42" s="35"/>
+      <c r="T42" s="35"/>
+      <c r="U42" s="35"/>
+      <c r="V42" s="35"/>
+      <c r="W42" s="35"/>
+      <c r="X42" s="35"/>
+      <c r="Y42" s="35"/>
+      <c r="Z42" s="35"/>
+      <c r="AA42" s="35"/>
+      <c r="AB42" s="35"/>
+      <c r="AC42" s="35"/>
+      <c r="AD42" s="35"/>
+      <c r="AE42" s="35"/>
+      <c r="AF42" s="35"/>
     </row>
     <row r="43" spans="1:32">
       <c r="A43" s="16" t="s">
@@ -9959,59 +10011,59 @@
       </c>
       <c r="O45" s="18"/>
     </row>
-    <row r="46" spans="1:32">
-      <c r="A46" s="17">
+    <row r="46" spans="1:32" s="34" customFormat="1">
+      <c r="A46" s="33">
         <v>3</v>
       </c>
-      <c r="B46" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="18" t="s">
+      <c r="B46" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C46" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="D46" s="18" t="s">
+      <c r="D46" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F46" s="18" t="s">
+      <c r="F46" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G46" s="18"/>
-      <c r="J46" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K46" s="18" t="s">
+      <c r="G46" s="32"/>
+      <c r="J46" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="K46" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="L46" s="18" t="s">
+      <c r="L46" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="M46" s="18" t="s">
+      <c r="M46" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="N46" s="18" t="s">
+      <c r="N46" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="O46" s="20"/>
-      <c r="P46" s="20"/>
-      <c r="Q46" s="20"/>
-      <c r="R46" s="20"/>
-      <c r="S46" s="20"/>
-      <c r="T46" s="20"/>
-      <c r="U46" s="20"/>
-      <c r="V46" s="20"/>
-      <c r="W46" s="20"/>
-      <c r="X46" s="20"/>
-      <c r="Y46" s="20"/>
-      <c r="Z46" s="20"/>
-      <c r="AA46" s="20"/>
-      <c r="AB46" s="20"/>
-      <c r="AC46" s="20"/>
-      <c r="AD46" s="20"/>
-      <c r="AE46" s="20"/>
-      <c r="AF46" s="20"/>
+      <c r="O46" s="35"/>
+      <c r="P46" s="35"/>
+      <c r="Q46" s="35"/>
+      <c r="R46" s="35"/>
+      <c r="S46" s="35"/>
+      <c r="T46" s="35"/>
+      <c r="U46" s="35"/>
+      <c r="V46" s="35"/>
+      <c r="W46" s="35"/>
+      <c r="X46" s="35"/>
+      <c r="Y46" s="35"/>
+      <c r="Z46" s="35"/>
+      <c r="AA46" s="35"/>
+      <c r="AB46" s="35"/>
+      <c r="AC46" s="35"/>
+      <c r="AD46" s="35"/>
+      <c r="AE46" s="35"/>
+      <c r="AF46" s="35"/>
     </row>
     <row r="47" spans="1:32">
       <c r="A47" s="16" t="s">
@@ -10104,59 +10156,59 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:32">
-      <c r="A50" s="18">
+    <row r="50" spans="1:32" s="34" customFormat="1">
+      <c r="A50" s="32">
         <v>3</v>
       </c>
-      <c r="B50" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C50" s="18" t="s">
+      <c r="B50" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C50" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="D50" s="18" t="s">
+      <c r="D50" s="32" t="s">
         <v>210</v>
       </c>
-      <c r="E50" s="18" t="s">
+      <c r="E50" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F50" s="18" t="s">
+      <c r="F50" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G50" s="18"/>
-      <c r="J50" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K50" s="18" t="s">
+      <c r="G50" s="32"/>
+      <c r="J50" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="K50" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="L50" s="18" t="s">
+      <c r="L50" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="M50" s="18" t="s">
+      <c r="M50" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="N50" s="18" t="s">
+      <c r="N50" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="O50" s="20"/>
-      <c r="P50" s="20"/>
-      <c r="Q50" s="20"/>
-      <c r="R50" s="20"/>
-      <c r="S50" s="20"/>
-      <c r="T50" s="20"/>
-      <c r="U50" s="20"/>
-      <c r="V50" s="20"/>
-      <c r="W50" s="20"/>
-      <c r="X50" s="20"/>
-      <c r="Y50" s="20"/>
-      <c r="Z50" s="20"/>
-      <c r="AA50" s="20"/>
-      <c r="AB50" s="20"/>
-      <c r="AC50" s="20"/>
-      <c r="AD50" s="20"/>
-      <c r="AE50" s="20"/>
-      <c r="AF50" s="20"/>
+      <c r="O50" s="35"/>
+      <c r="P50" s="35"/>
+      <c r="Q50" s="35"/>
+      <c r="R50" s="35"/>
+      <c r="S50" s="35"/>
+      <c r="T50" s="35"/>
+      <c r="U50" s="35"/>
+      <c r="V50" s="35"/>
+      <c r="W50" s="35"/>
+      <c r="X50" s="35"/>
+      <c r="Y50" s="35"/>
+      <c r="Z50" s="35"/>
+      <c r="AA50" s="35"/>
+      <c r="AB50" s="35"/>
+      <c r="AC50" s="35"/>
+      <c r="AD50" s="35"/>
+      <c r="AE50" s="35"/>
+      <c r="AF50" s="35"/>
     </row>
     <row r="51" spans="1:32">
       <c r="A51" s="16" t="s">
@@ -10249,59 +10301,59 @@
         <v>57</v>
       </c>
     </row>
-    <row r="54" spans="1:32">
-      <c r="A54" s="18">
+    <row r="54" spans="1:32" s="34" customFormat="1">
+      <c r="A54" s="32">
         <v>3</v>
       </c>
-      <c r="B54" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C54" s="18" t="s">
+      <c r="B54" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C54" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="D54" s="18" t="s">
+      <c r="D54" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="E54" s="18" t="s">
+      <c r="E54" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F54" s="18" t="s">
+      <c r="F54" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G54" s="18"/>
-      <c r="J54" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K54" s="18" t="s">
+      <c r="G54" s="32"/>
+      <c r="J54" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="K54" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="L54" s="18" t="s">
+      <c r="L54" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="M54" s="18" t="s">
+      <c r="M54" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="N54" s="18" t="s">
+      <c r="N54" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="O54" s="20"/>
-      <c r="P54" s="20"/>
-      <c r="Q54" s="20"/>
-      <c r="R54" s="20"/>
-      <c r="S54" s="20"/>
-      <c r="T54" s="20"/>
-      <c r="U54" s="20"/>
-      <c r="V54" s="20"/>
-      <c r="W54" s="20"/>
-      <c r="X54" s="20"/>
-      <c r="Y54" s="20"/>
-      <c r="Z54" s="20"/>
-      <c r="AA54" s="20"/>
-      <c r="AB54" s="20"/>
-      <c r="AC54" s="20"/>
-      <c r="AD54" s="20"/>
-      <c r="AE54" s="20"/>
-      <c r="AF54" s="20"/>
+      <c r="O54" s="35"/>
+      <c r="P54" s="35"/>
+      <c r="Q54" s="35"/>
+      <c r="R54" s="35"/>
+      <c r="S54" s="35"/>
+      <c r="T54" s="35"/>
+      <c r="U54" s="35"/>
+      <c r="V54" s="35"/>
+      <c r="W54" s="35"/>
+      <c r="X54" s="35"/>
+      <c r="Y54" s="35"/>
+      <c r="Z54" s="35"/>
+      <c r="AA54" s="35"/>
+      <c r="AB54" s="35"/>
+      <c r="AC54" s="35"/>
+      <c r="AD54" s="35"/>
+      <c r="AE54" s="35"/>
+      <c r="AF54" s="35"/>
     </row>
     <row r="55" spans="1:32">
       <c r="A55" s="16" t="s">
@@ -16736,190 +16788,190 @@
         <v>42</v>
       </c>
     </row>
-    <row r="57" spans="1:19">
-      <c r="A57" s="18">
+    <row r="57" spans="1:19" s="34" customFormat="1">
+      <c r="A57" s="32">
         <v>1</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C57" s="18" t="s">
+      <c r="C57" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="D57" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E57" s="18" t="s">
+      <c r="D57" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E57" s="32" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="58" spans="1:19">
-      <c r="A58" s="18">
+    <row r="58" spans="1:19" s="34" customFormat="1">
+      <c r="A58" s="32">
         <v>2</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C58" s="18" t="s">
+      <c r="C58" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="D58" s="18" t="s">
+      <c r="D58" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="59" spans="1:19">
-      <c r="A59" s="18">
+    <row r="59" spans="1:19" s="34" customFormat="1">
+      <c r="A59" s="32">
         <v>3</v>
       </c>
-      <c r="B59" s="18" t="s">
+      <c r="B59" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C59" s="18" t="s">
+      <c r="C59" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="D59" s="18" t="s">
+      <c r="D59" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="18" t="s">
+      <c r="E59" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="60" spans="1:19">
-      <c r="A60" s="18">
+    <row r="60" spans="1:19" s="34" customFormat="1">
+      <c r="A60" s="32">
         <v>4</v>
       </c>
-      <c r="B60" s="18" t="s">
+      <c r="B60" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C60" s="18" t="s">
+      <c r="C60" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="D60" s="18" t="s">
+      <c r="D60" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E60" s="18" t="s">
+      <c r="E60" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="61" spans="1:19">
-      <c r="A61" s="18">
+    <row r="61" spans="1:19" s="34" customFormat="1">
+      <c r="A61" s="32">
         <v>5</v>
       </c>
-      <c r="B61" s="18" t="s">
+      <c r="B61" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C61" s="18" t="s">
+      <c r="C61" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="D61" s="18" t="s">
+      <c r="D61" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E61" s="18" t="s">
+      <c r="E61" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="62" spans="1:19">
-      <c r="A62" s="18">
+    <row r="62" spans="1:19" s="34" customFormat="1">
+      <c r="A62" s="32">
         <v>6</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C62" s="18" t="s">
+      <c r="C62" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="D62" s="18" t="s">
+      <c r="D62" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E62" s="18" t="s">
+      <c r="E62" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="63" spans="1:19">
-      <c r="A63" s="18">
+    <row r="63" spans="1:19" s="34" customFormat="1">
+      <c r="A63" s="32">
         <v>7</v>
       </c>
-      <c r="B63" s="18" t="s">
+      <c r="B63" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C63" s="18" t="s">
+      <c r="C63" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="D63" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E63" s="18" t="s">
+      <c r="D63" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E63" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="64" spans="1:19">
-      <c r="A64" s="18">
+    <row r="64" spans="1:19" s="34" customFormat="1">
+      <c r="A64" s="32">
         <v>8</v>
       </c>
-      <c r="B64" s="18" t="s">
+      <c r="B64" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="32" t="s">
         <v>246</v>
       </c>
-      <c r="D64" s="18" t="s">
+      <c r="D64" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E64" s="18" t="s">
+      <c r="E64" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="65" spans="1:19">
-      <c r="A65" s="18">
+    <row r="65" spans="1:19" s="34" customFormat="1">
+      <c r="A65" s="32">
         <v>9</v>
       </c>
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C65" s="18" t="s">
+      <c r="C65" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="D65" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E65" s="18" t="s">
+      <c r="D65" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E65" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="66" spans="1:19">
-      <c r="A66" s="18">
+    <row r="66" spans="1:19" s="34" customFormat="1">
+      <c r="A66" s="32">
         <v>10</v>
       </c>
-      <c r="B66" s="18" t="s">
+      <c r="B66" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C66" s="18" t="s">
+      <c r="C66" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="D66" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E66" s="18" t="s">
+      <c r="D66" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E66" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="67" spans="1:19">
-      <c r="A67" s="18">
+    <row r="67" spans="1:19" s="34" customFormat="1">
+      <c r="A67" s="32">
         <v>11</v>
       </c>
-      <c r="B67" s="18" t="s">
+      <c r="B67" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="C67" s="18" t="s">
+      <c r="C67" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="D67" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E67" s="18" t="s">
+      <c r="D67" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E67" s="32" t="s">
         <v>234</v>
       </c>
     </row>
@@ -17000,54 +17052,54 @@
         <v>232</v>
       </c>
     </row>
-    <row r="72" spans="1:19">
-      <c r="A72" s="18">
+    <row r="72" spans="1:19" s="34" customFormat="1">
+      <c r="A72" s="32">
         <v>3</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C72" s="18" t="s">
+      <c r="C72" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="D72" s="18" t="s">
+      <c r="D72" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E72" s="18" t="s">
+      <c r="E72" s="32" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="73" spans="1:19">
-      <c r="A73" s="18">
+    <row r="73" spans="1:19" s="34" customFormat="1">
+      <c r="A73" s="32">
         <v>4</v>
       </c>
-      <c r="B73" s="18" t="s">
+      <c r="B73" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C73" s="18" t="s">
+      <c r="C73" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="D73" s="18" t="s">
+      <c r="D73" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E73" s="18" t="s">
+      <c r="E73" s="32" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="74" spans="1:19">
-      <c r="A74" s="18">
+    <row r="74" spans="1:19" s="34" customFormat="1">
+      <c r="A74" s="32">
         <v>5</v>
       </c>
-      <c r="B74" s="18" t="s">
+      <c r="B74" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C74" s="18" t="s">
+      <c r="C74" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="D74" s="18" t="s">
+      <c r="D74" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E74" s="18" t="s">
+      <c r="E74" s="32" t="s">
         <v>232</v>
       </c>
     </row>
@@ -17170,112 +17222,129 @@
         <v>232</v>
       </c>
     </row>
-    <row r="82" spans="1:19">
-      <c r="A82" s="18">
+    <row r="82" spans="1:19" s="34" customFormat="1">
+      <c r="A82" s="32">
         <v>13</v>
       </c>
-      <c r="B82" s="18" t="s">
+      <c r="B82" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C82" s="18" t="s">
+      <c r="C82" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="D82" s="18" t="s">
+      <c r="D82" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="E82" s="18" t="s">
+      <c r="E82" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="83" spans="1:19">
-      <c r="A83" s="18">
+    <row r="83" spans="1:19" s="34" customFormat="1">
+      <c r="A83" s="32">
         <v>14</v>
       </c>
-      <c r="B83" s="18" t="s">
+      <c r="B83" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C83" s="18" t="s">
+      <c r="C83" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="D83" s="18" t="s">
+      <c r="D83" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="E83" s="18" t="s">
+      <c r="E83" s="32" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="84" spans="1:19">
-      <c r="A84" s="18">
+    <row r="84" spans="1:19" s="34" customFormat="1">
+      <c r="A84" s="32">
         <v>15</v>
       </c>
-      <c r="B84" s="18" t="s">
+      <c r="B84" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C84" s="18" t="s">
+      <c r="C84" s="32" t="s">
         <v>134</v>
       </c>
-      <c r="D84" s="18" t="s">
+      <c r="D84" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="E84" s="18" t="s">
+      <c r="E84" s="32" t="s">
         <v>234</v>
       </c>
     </row>
+    <row r="85" spans="1:19">
+      <c r="A85" s="22"/>
+      <c r="B85" s="22"/>
+      <c r="C85" s="22"/>
+      <c r="D85" s="22"/>
+      <c r="E85" s="22"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="22"/>
+      <c r="I85" s="17"/>
+      <c r="J85" s="17"/>
+      <c r="K85" s="17"/>
+      <c r="L85" s="17"/>
+      <c r="M85" s="17"/>
+      <c r="N85" s="17"/>
+      <c r="O85" s="17"/>
+      <c r="P85" s="17"/>
+      <c r="Q85" s="17"/>
+      <c r="R85" s="17"/>
+      <c r="S85" s="17"/>
+    </row>
     <row r="86" spans="1:19">
-      <c r="A86" s="22"/>
-      <c r="B86" s="22"/>
-      <c r="C86" s="22"/>
-      <c r="D86" s="22"/>
-      <c r="E86" s="22"/>
-      <c r="F86" s="22"/>
-      <c r="G86" s="22"/>
-      <c r="I86" s="17"/>
-      <c r="J86" s="17"/>
-      <c r="K86" s="17"/>
-      <c r="L86" s="17"/>
-      <c r="M86" s="17"/>
-      <c r="N86" s="17"/>
-      <c r="O86" s="17"/>
-      <c r="P86" s="17"/>
-      <c r="Q86" s="17"/>
-      <c r="R86" s="17"/>
-      <c r="S86" s="17"/>
+      <c r="A86" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B86" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="C86" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="D86" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="E86" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="F86" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="G86" s="21" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="87" spans="1:19">
-      <c r="A87" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B87" s="21" t="s">
-        <v>225</v>
-      </c>
-      <c r="C87" s="21" t="s">
-        <v>226</v>
-      </c>
-      <c r="D87" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="E87" s="21" t="s">
-        <v>228</v>
-      </c>
-      <c r="F87" s="21" t="s">
-        <v>229</v>
-      </c>
-      <c r="G87" s="21" t="s">
-        <v>42</v>
+      <c r="A87" s="18">
+        <v>2</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="D87" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="E87" s="18" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="88" spans="1:19">
       <c r="A88" s="18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B88" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C88" s="18" t="s">
-        <v>106</v>
+        <v>172</v>
       </c>
       <c r="D88" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="E88" s="18" t="s">
         <v>234</v>
@@ -17283,13 +17352,13 @@
     </row>
     <row r="89" spans="1:19">
       <c r="A89" s="18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B89" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D89" s="18" t="s">
         <v>120</v>
@@ -17300,16 +17369,16 @@
     </row>
     <row r="90" spans="1:19">
       <c r="A90" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B90" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C90" s="18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D90" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="E90" s="18" t="s">
         <v>234</v>
@@ -17317,13 +17386,13 @@
     </row>
     <row r="91" spans="1:19">
       <c r="A91" s="18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B91" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C91" s="18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D91" s="18" t="s">
         <v>50</v>
@@ -17334,13 +17403,13 @@
     </row>
     <row r="92" spans="1:19">
       <c r="A92" s="18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B92" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C92" s="18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D92" s="18" t="s">
         <v>50</v>
@@ -17351,13 +17420,13 @@
     </row>
     <row r="93" spans="1:19">
       <c r="A93" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B93" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C93" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D93" s="18" t="s">
         <v>50</v>
@@ -17367,38 +17436,41 @@
       </c>
     </row>
     <row r="94" spans="1:19">
-      <c r="A94" s="18">
-        <v>8</v>
+      <c r="A94" s="17">
+        <v>9</v>
       </c>
       <c r="B94" s="18" t="s">
         <v>25</v>
       </c>
       <c r="C94" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D94" s="18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E94" s="18" t="s">
         <v>234</v>
       </c>
+      <c r="F94" s="22"/>
+      <c r="G94" s="22"/>
+      <c r="I94" s="17"/>
+      <c r="J94" s="17"/>
+      <c r="K94" s="17"/>
+      <c r="L94" s="17"/>
+      <c r="M94" s="17"/>
+      <c r="N94" s="17"/>
+      <c r="O94" s="17"/>
+      <c r="P94" s="17"/>
+      <c r="Q94" s="17"/>
+      <c r="R94" s="17"/>
+      <c r="S94" s="17"/>
     </row>
     <row r="95" spans="1:19">
-      <c r="A95" s="17">
-        <v>9</v>
-      </c>
-      <c r="B95" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C95" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="D95" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E95" s="18" t="s">
-        <v>234</v>
-      </c>
+      <c r="A95" s="17"/>
+      <c r="B95" s="18"/>
+      <c r="C95" s="18"/>
+      <c r="D95" s="18"/>
+      <c r="E95" s="18"/>
       <c r="F95" s="22"/>
       <c r="G95" s="22"/>
       <c r="I95" s="17"/>
@@ -17855,21 +17927,25 @@
     <tabColor rgb="FF351C75"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AF936"/>
+  <dimension ref="A1:AF940"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2.33203125" customWidth="1"/>
-    <col min="10" max="10" width="15.88671875" customWidth="1"/>
-    <col min="11" max="11" width="24.33203125" customWidth="1"/>
-    <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="21" customWidth="1"/>
-    <col min="14" max="14" width="19.88671875" customWidth="1"/>
-    <col min="15" max="16" width="17" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="24.88671875" customWidth="1"/>
     <col min="20" max="20" width="23.109375" customWidth="1"/>
     <col min="21" max="21" width="17.33203125" customWidth="1"/>
@@ -17877,23 +17953,23 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="23"/>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="39" t="s">
         <v>253</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="J1" s="34" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="J1" s="41" t="s">
         <v>254</v>
       </c>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
       <c r="P1" s="13"/>
     </row>
     <row r="2" spans="1:16">
@@ -17941,22 +18017,22 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="17"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
+    <row r="3" spans="1:16" s="38" customFormat="1">
+      <c r="A3" s="36"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="17"/>
@@ -18593,60 +18669,60 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:32">
-      <c r="A22" s="20"/>
-      <c r="B22" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="18" t="s">
+    <row r="22" spans="1:32" s="34" customFormat="1">
+      <c r="A22" s="35"/>
+      <c r="B22" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="20"/>
-      <c r="M22" s="20"/>
-      <c r="N22" s="20"/>
-      <c r="O22" s="20"/>
-      <c r="P22" s="20"/>
-      <c r="Q22" s="20"/>
-      <c r="R22" s="20"/>
-      <c r="S22" s="20"/>
-      <c r="T22" s="20"/>
-      <c r="U22" s="20"/>
-      <c r="V22" s="20"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="20"/>
-      <c r="Y22" s="20"/>
-      <c r="Z22" s="20"/>
-      <c r="AA22" s="20"/>
-      <c r="AB22" s="20"/>
-      <c r="AC22" s="20"/>
-      <c r="AD22" s="20"/>
-      <c r="AE22" s="20"/>
-      <c r="AF22" s="20"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="35"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="35"/>
+      <c r="R22" s="35"/>
+      <c r="S22" s="35"/>
+      <c r="T22" s="35"/>
+      <c r="U22" s="35"/>
+      <c r="V22" s="35"/>
+      <c r="W22" s="35"/>
+      <c r="X22" s="35"/>
+      <c r="Y22" s="35"/>
+      <c r="Z22" s="35"/>
+      <c r="AA22" s="35"/>
+      <c r="AB22" s="35"/>
+      <c r="AC22" s="35"/>
+      <c r="AD22" s="35"/>
+      <c r="AE22" s="35"/>
+      <c r="AF22" s="35"/>
     </row>
     <row r="23" spans="1:32">
       <c r="A23" s="17"/>
-      <c r="B23" s="3"/>
+      <c r="B23" s="37"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="J23" s="3"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
@@ -19286,98 +19362,100 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:32">
-      <c r="A42" s="20"/>
-      <c r="B42" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="18" t="s">
+    <row r="42" spans="1:32" s="34" customFormat="1">
+      <c r="A42" s="35"/>
+      <c r="B42" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F42" s="18" t="s">
+      <c r="F42" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="20"/>
-      <c r="P42" s="20"/>
-      <c r="Q42" s="20"/>
-      <c r="R42" s="20"/>
-      <c r="S42" s="20"/>
-      <c r="T42" s="20"/>
-      <c r="U42" s="20"/>
-      <c r="V42" s="20"/>
-      <c r="W42" s="20"/>
-      <c r="X42" s="20"/>
-      <c r="Y42" s="20"/>
-      <c r="Z42" s="20"/>
-      <c r="AA42" s="20"/>
-      <c r="AB42" s="20"/>
-      <c r="AC42" s="20"/>
-      <c r="AD42" s="20"/>
-      <c r="AE42" s="20"/>
-      <c r="AF42" s="20"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="35"/>
+      <c r="I42" s="35"/>
+      <c r="J42" s="35"/>
+      <c r="K42" s="35"/>
+      <c r="L42" s="35"/>
+      <c r="M42" s="35"/>
+      <c r="N42" s="35"/>
+      <c r="O42" s="35"/>
+      <c r="P42" s="35"/>
+      <c r="Q42" s="35"/>
+      <c r="R42" s="35"/>
+      <c r="S42" s="35"/>
+      <c r="T42" s="35"/>
+      <c r="U42" s="35"/>
+      <c r="V42" s="35"/>
+      <c r="W42" s="35"/>
+      <c r="X42" s="35"/>
+      <c r="Y42" s="35"/>
+      <c r="Z42" s="35"/>
+      <c r="AA42" s="35"/>
+      <c r="AB42" s="35"/>
+      <c r="AC42" s="35"/>
+      <c r="AD42" s="35"/>
+      <c r="AE42" s="35"/>
+      <c r="AF42" s="35"/>
     </row>
     <row r="43" spans="1:32">
-      <c r="A43" s="17"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-      <c r="N43" s="3"/>
-      <c r="O43" s="3"/>
-      <c r="P43" s="3"/>
+      <c r="A43" s="20"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="20"/>
+      <c r="K43" s="20"/>
+      <c r="L43" s="20"/>
+      <c r="M43" s="20"/>
+      <c r="N43" s="20"/>
+      <c r="O43" s="20"/>
+      <c r="P43" s="20"/>
+      <c r="Q43" s="20"/>
+      <c r="R43" s="20"/>
+      <c r="S43" s="20"/>
+      <c r="T43" s="20"/>
+      <c r="U43" s="20"/>
+      <c r="V43" s="20"/>
+      <c r="W43" s="20"/>
+      <c r="X43" s="20"/>
+      <c r="Y43" s="20"/>
+      <c r="Z43" s="20"/>
+      <c r="AA43" s="20"/>
+      <c r="AB43" s="20"/>
+      <c r="AC43" s="20"/>
+      <c r="AD43" s="20"/>
+      <c r="AE43" s="20"/>
+      <c r="AF43" s="20"/>
     </row>
     <row r="44" spans="1:32">
       <c r="A44" s="17"/>
-      <c r="B44" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D44" s="20" t="s">
-        <v>238</v>
-      </c>
-      <c r="E44" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="F44" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="G44" s="20" t="s">
-        <v>233</v>
-      </c>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20" t="s">
-        <v>257</v>
-      </c>
-      <c r="K44" s="20"/>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
-      <c r="N44" s="20"/>
-      <c r="O44" s="20"/>
-      <c r="P44" s="20"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+      <c r="P44" s="3"/>
     </row>
     <row r="45" spans="1:32">
       <c r="A45" s="17"/>
@@ -19391,12 +19469,14 @@
         <v>238</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>239</v>
+        <v>256</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>240</v>
-      </c>
-      <c r="G45" s="20"/>
+        <v>57</v>
+      </c>
+      <c r="G45" s="20" t="s">
+        <v>233</v>
+      </c>
       <c r="H45" s="20"/>
       <c r="I45" s="20"/>
       <c r="J45" s="20" t="s">
@@ -19421,10 +19501,10 @@
         <v>238</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>50</v>
+        <v>240</v>
       </c>
       <c r="G46" s="20"/>
       <c r="H46" s="20"/>
@@ -19451,13 +19531,13 @@
         <v>238</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F47" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="G47" s="26"/>
-      <c r="H47" s="27"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
       <c r="I47" s="20"/>
       <c r="J47" s="20" t="s">
         <v>257</v>
@@ -19481,13 +19561,13 @@
         <v>238</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F48" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="G48" s="19"/>
-      <c r="H48" s="19"/>
+      <c r="G48" s="26"/>
+      <c r="H48" s="27"/>
       <c r="I48" s="20"/>
       <c r="J48" s="20" t="s">
         <v>257</v>
@@ -19511,7 +19591,7 @@
         <v>238</v>
       </c>
       <c r="E49" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F49" s="19" t="s">
         <v>50</v>
@@ -19541,10 +19621,10 @@
         <v>238</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="G50" s="19"/>
       <c r="H50" s="19"/>
@@ -19571,10 +19651,10 @@
         <v>238</v>
       </c>
       <c r="E51" s="19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G51" s="19"/>
       <c r="H51" s="19"/>
@@ -19601,10 +19681,10 @@
         <v>238</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="G52" s="19"/>
       <c r="H52" s="19"/>
@@ -19631,7 +19711,7 @@
         <v>238</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F53" s="19" t="s">
         <v>57</v>
@@ -19661,7 +19741,7 @@
         <v>238</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F54" s="19" t="s">
         <v>57</v>
@@ -19691,10 +19771,10 @@
         <v>238</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G55" s="19"/>
       <c r="H55" s="19"/>
@@ -19710,88 +19790,85 @@
       <c r="P55" s="20"/>
     </row>
     <row r="56" spans="1:32">
-      <c r="A56" s="20"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
+      <c r="A56" s="17"/>
+      <c r="B56" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C56" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D56" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E56" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="F56" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19"/>
       <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
+      <c r="J56" s="20" t="s">
+        <v>257</v>
+      </c>
       <c r="K56" s="20"/>
       <c r="L56" s="20"/>
       <c r="M56" s="20"/>
       <c r="N56" s="20"/>
       <c r="O56" s="20"/>
       <c r="P56" s="20"/>
-      <c r="Q56" s="20"/>
-      <c r="R56" s="20"/>
-      <c r="S56" s="20"/>
-      <c r="T56" s="20"/>
-      <c r="U56" s="20"/>
-      <c r="V56" s="20"/>
-      <c r="W56" s="20"/>
-      <c r="X56" s="20"/>
-      <c r="Y56" s="20"/>
-      <c r="Z56" s="20"/>
-      <c r="AA56" s="20"/>
-      <c r="AB56" s="20"/>
-      <c r="AC56" s="20"/>
-      <c r="AD56" s="20"/>
-      <c r="AE56" s="20"/>
-      <c r="AF56" s="20"/>
     </row>
     <row r="57" spans="1:32">
-      <c r="A57" s="17"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3"/>
-      <c r="J57" s="3"/>
-      <c r="K57" s="3"/>
-      <c r="L57" s="3"/>
-      <c r="M57" s="3"/>
-      <c r="N57" s="3"/>
-      <c r="O57" s="3"/>
-      <c r="P57" s="3"/>
+      <c r="A57" s="20"/>
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20"/>
+      <c r="M57" s="20"/>
+      <c r="N57" s="20"/>
+      <c r="O57" s="20"/>
+      <c r="P57" s="20"/>
+      <c r="Q57" s="20"/>
+      <c r="R57" s="20"/>
+      <c r="S57" s="20"/>
+      <c r="T57" s="20"/>
+      <c r="U57" s="20"/>
+      <c r="V57" s="20"/>
+      <c r="W57" s="20"/>
+      <c r="X57" s="20"/>
+      <c r="Y57" s="20"/>
+      <c r="Z57" s="20"/>
+      <c r="AA57" s="20"/>
+      <c r="AB57" s="20"/>
+      <c r="AC57" s="20"/>
+      <c r="AD57" s="20"/>
+      <c r="AE57" s="20"/>
+      <c r="AF57" s="20"/>
     </row>
     <row r="58" spans="1:32">
       <c r="A58" s="17"/>
-      <c r="B58" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C58" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D58" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="E58" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="F58" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J58" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K58" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L58" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="M58" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="N58" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="3"/>
+      <c r="N58" s="3"/>
+      <c r="O58" s="3"/>
+      <c r="P58" s="3"/>
     </row>
     <row r="59" spans="1:32">
       <c r="A59" s="17"/>
@@ -19805,10 +19882,10 @@
         <v>250</v>
       </c>
       <c r="E59" s="18" t="s">
-        <v>142</v>
+        <v>174</v>
       </c>
       <c r="F59" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J59" s="17" t="s">
         <v>47</v>
@@ -19820,10 +19897,10 @@
         <v>217</v>
       </c>
       <c r="M59" s="18" t="s">
-        <v>142</v>
+        <v>49</v>
       </c>
       <c r="N59" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="60" spans="1:32">
@@ -19838,7 +19915,7 @@
         <v>250</v>
       </c>
       <c r="E60" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F60" s="18" t="s">
         <v>57</v>
@@ -19853,7 +19930,7 @@
         <v>217</v>
       </c>
       <c r="M60" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N60" s="18" t="s">
         <v>57</v>
@@ -19871,7 +19948,7 @@
         <v>250</v>
       </c>
       <c r="E61" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F61" s="18" t="s">
         <v>57</v>
@@ -19886,7 +19963,7 @@
         <v>217</v>
       </c>
       <c r="M61" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N61" s="18" t="s">
         <v>57</v>
@@ -19904,7 +19981,7 @@
         <v>250</v>
       </c>
       <c r="E62" s="18" t="s">
-        <v>252</v>
+        <v>144</v>
       </c>
       <c r="F62" s="18" t="s">
         <v>57</v>
@@ -19916,10 +19993,10 @@
         <v>204</v>
       </c>
       <c r="L62" s="18" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M62" s="18" t="s">
-        <v>56</v>
+        <v>144</v>
       </c>
       <c r="N62" s="18" t="s">
         <v>57</v>
@@ -19937,10 +20014,10 @@
         <v>250</v>
       </c>
       <c r="E63" s="18" t="s">
-        <v>145</v>
+        <v>252</v>
       </c>
       <c r="F63" s="18" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="J63" s="17" t="s">
         <v>47</v>
@@ -19949,13 +20026,13 @@
         <v>204</v>
       </c>
       <c r="L63" s="18" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="M63" s="18" t="s">
-        <v>145</v>
+        <v>56</v>
       </c>
       <c r="N63" s="18" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
     </row>
     <row r="64" spans="1:32">
@@ -19970,7 +20047,7 @@
         <v>250</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F64" s="18" t="s">
         <v>130</v>
@@ -19985,7 +20062,7 @@
         <v>217</v>
       </c>
       <c r="M64" s="18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="N64" s="18" t="s">
         <v>130</v>
@@ -20003,10 +20080,10 @@
         <v>250</v>
       </c>
       <c r="E65" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F65" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="J65" s="17" t="s">
         <v>47</v>
@@ -20018,10 +20095,10 @@
         <v>217</v>
       </c>
       <c r="M65" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N65" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:32">
@@ -20036,7 +20113,7 @@
         <v>250</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F66" s="18" t="s">
         <v>50</v>
@@ -20051,7 +20128,7 @@
         <v>217</v>
       </c>
       <c r="M66" s="18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N66" s="18" t="s">
         <v>50</v>
@@ -20069,10 +20146,10 @@
         <v>250</v>
       </c>
       <c r="E67" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F67" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J67" s="17" t="s">
         <v>47</v>
@@ -20084,10 +20161,10 @@
         <v>217</v>
       </c>
       <c r="M67" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N67" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="68" spans="1:32">
@@ -20102,10 +20179,10 @@
         <v>250</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F68" s="18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="J68" s="17" t="s">
         <v>47</v>
@@ -20117,10 +20194,10 @@
         <v>217</v>
       </c>
       <c r="M68" s="18" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N68" s="18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="69" spans="1:32">
@@ -20135,7 +20212,7 @@
         <v>250</v>
       </c>
       <c r="E69" s="18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F69" s="18" t="s">
         <v>50</v>
@@ -20150,7 +20227,7 @@
         <v>217</v>
       </c>
       <c r="M69" s="18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="N69" s="18" t="s">
         <v>50</v>
@@ -20168,10 +20245,10 @@
         <v>250</v>
       </c>
       <c r="E70" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F70" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J70" s="17" t="s">
         <v>47</v>
@@ -20183,10 +20260,10 @@
         <v>217</v>
       </c>
       <c r="M70" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N70" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:32">
@@ -20201,7 +20278,7 @@
         <v>250</v>
       </c>
       <c r="E71" s="18" t="s">
-        <v>92</v>
+        <v>153</v>
       </c>
       <c r="F71" s="18" t="s">
         <v>57</v>
@@ -20216,14 +20293,14 @@
         <v>217</v>
       </c>
       <c r="M71" s="18" t="s">
-        <v>92</v>
+        <v>153</v>
       </c>
       <c r="N71" s="18" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="72" spans="1:32">
-      <c r="A72" s="20"/>
+      <c r="A72" s="17"/>
       <c r="B72" s="28" t="s">
         <v>47</v>
       </c>
@@ -20234,120 +20311,121 @@
         <v>250</v>
       </c>
       <c r="E72" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="F72" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="J72" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K72" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L72" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="M72" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="N72" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="73" spans="1:32" s="34" customFormat="1">
+      <c r="A73" s="35"/>
+      <c r="B73" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="C73" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="D73" s="32" t="s">
+        <v>250</v>
+      </c>
+      <c r="E73" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="F72" s="18" t="s">
+      <c r="F73" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="G72" s="20"/>
-      <c r="H72" s="20"/>
-      <c r="I72" s="20"/>
-      <c r="J72" s="20"/>
-      <c r="K72" s="20"/>
-      <c r="L72" s="20"/>
-      <c r="M72" s="20"/>
-      <c r="N72" s="20"/>
-      <c r="O72" s="20"/>
-      <c r="P72" s="20"/>
-      <c r="Q72" s="20"/>
-      <c r="R72" s="20"/>
-      <c r="S72" s="20"/>
-      <c r="T72" s="20"/>
-      <c r="U72" s="20"/>
-      <c r="V72" s="20"/>
-      <c r="W72" s="20"/>
-      <c r="X72" s="20"/>
-      <c r="Y72" s="20"/>
-      <c r="Z72" s="20"/>
-      <c r="AA72" s="20"/>
-      <c r="AB72" s="20"/>
-      <c r="AC72" s="20"/>
-      <c r="AD72" s="20"/>
-      <c r="AE72" s="20"/>
-      <c r="AF72" s="20"/>
-    </row>
-    <row r="73" spans="1:32">
-      <c r="A73" s="17"/>
-      <c r="B73" s="29"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
-      <c r="J73" s="3"/>
-      <c r="K73" s="3"/>
-      <c r="L73" s="3"/>
-      <c r="M73" s="3"/>
-      <c r="N73" s="3"/>
-      <c r="O73" s="3"/>
-      <c r="P73" s="3"/>
-    </row>
-    <row r="74" spans="1:32">
-      <c r="A74" s="17"/>
-      <c r="B74" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C74" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D74" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E74" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="F74" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J74" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K74" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L74" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="M74" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="N74" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="G73" s="35"/>
+      <c r="H73" s="35"/>
+      <c r="I73" s="35"/>
+      <c r="J73" s="35"/>
+      <c r="K73" s="35"/>
+      <c r="L73" s="35"/>
+      <c r="M73" s="35"/>
+      <c r="N73" s="35"/>
+      <c r="O73" s="35"/>
+      <c r="P73" s="35"/>
+      <c r="Q73" s="35"/>
+      <c r="R73" s="35"/>
+      <c r="S73" s="35"/>
+      <c r="T73" s="35"/>
+      <c r="U73" s="35"/>
+      <c r="V73" s="35"/>
+      <c r="W73" s="35"/>
+      <c r="X73" s="35"/>
+      <c r="Y73" s="35"/>
+      <c r="Z73" s="35"/>
+      <c r="AA73" s="35"/>
+      <c r="AB73" s="35"/>
+      <c r="AC73" s="35"/>
+      <c r="AD73" s="35"/>
+      <c r="AE73" s="35"/>
+      <c r="AF73" s="35"/>
+    </row>
+    <row r="74" spans="1:32" s="46" customFormat="1">
+      <c r="A74" s="44"/>
+      <c r="B74" s="45"/>
+      <c r="C74" s="44"/>
+      <c r="D74" s="44"/>
+      <c r="E74" s="44"/>
+      <c r="F74" s="44"/>
+      <c r="G74" s="44"/>
+      <c r="H74" s="44"/>
+      <c r="I74" s="44"/>
+      <c r="J74" s="44"/>
+      <c r="K74" s="44"/>
+      <c r="L74" s="44"/>
+      <c r="M74" s="44"/>
+      <c r="N74" s="44"/>
+      <c r="O74" s="44"/>
+      <c r="P74" s="44"/>
+      <c r="Q74" s="44"/>
+      <c r="R74" s="44"/>
+      <c r="S74" s="44"/>
+      <c r="T74" s="44"/>
+      <c r="U74" s="44"/>
+      <c r="V74" s="44"/>
+      <c r="W74" s="44"/>
+      <c r="X74" s="44"/>
+      <c r="Y74" s="44"/>
+      <c r="Z74" s="44"/>
+      <c r="AA74" s="44"/>
+      <c r="AB74" s="44"/>
+      <c r="AC74" s="44"/>
+      <c r="AD74" s="44"/>
+      <c r="AE74" s="44"/>
+      <c r="AF74" s="44"/>
     </row>
     <row r="75" spans="1:32">
       <c r="A75" s="17"/>
-      <c r="B75" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C75" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D75" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E75" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="F75" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J75" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K75" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L75" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="M75" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="N75" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="B75" s="29"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="3"/>
     </row>
     <row r="76" spans="1:32">
       <c r="A76" s="17"/>
@@ -20361,10 +20439,10 @@
         <v>25</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="F76" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J76" s="17" t="s">
         <v>47</v>
@@ -20376,10 +20454,10 @@
         <v>220</v>
       </c>
       <c r="M76" s="18" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="N76" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="77" spans="1:32">
@@ -20394,10 +20472,10 @@
         <v>25</v>
       </c>
       <c r="E77" s="18" t="s">
-        <v>173</v>
+        <v>106</v>
       </c>
       <c r="F77" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J77" s="17" t="s">
         <v>47</v>
@@ -20409,10 +20487,10 @@
         <v>220</v>
       </c>
       <c r="M77" s="18" t="s">
-        <v>173</v>
+        <v>106</v>
       </c>
       <c r="N77" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="78" spans="1:32">
@@ -20427,10 +20505,10 @@
         <v>25</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F78" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="J78" s="17" t="s">
         <v>47</v>
@@ -20442,10 +20520,10 @@
         <v>220</v>
       </c>
       <c r="M78" s="18" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="N78" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="79" spans="1:32">
@@ -20460,10 +20538,10 @@
         <v>25</v>
       </c>
       <c r="E79" s="18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F79" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="J79" s="17" t="s">
         <v>47</v>
@@ -20475,10 +20553,10 @@
         <v>220</v>
       </c>
       <c r="M79" s="18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="N79" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="80" spans="1:32">
@@ -20493,7 +20571,7 @@
         <v>25</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F80" s="18" t="s">
         <v>50</v>
@@ -20508,7 +20586,7 @@
         <v>220</v>
       </c>
       <c r="M80" s="18" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="N80" s="18" t="s">
         <v>50</v>
@@ -20526,7 +20604,7 @@
         <v>25</v>
       </c>
       <c r="E81" s="18" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F81" s="18" t="s">
         <v>50</v>
@@ -20541,7 +20619,7 @@
         <v>220</v>
       </c>
       <c r="M81" s="18" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="N81" s="18" t="s">
         <v>50</v>
@@ -20559,10 +20637,10 @@
         <v>25</v>
       </c>
       <c r="E82" s="18" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F82" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J82" s="17" t="s">
         <v>47</v>
@@ -20574,14 +20652,14 @@
         <v>220</v>
       </c>
       <c r="M82" s="18" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="N82" s="18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83" spans="1:32">
-      <c r="A83" s="20"/>
+      <c r="A83" s="17"/>
       <c r="B83" s="28" t="s">
         <v>47</v>
       </c>
@@ -20592,153 +20670,154 @@
         <v>25</v>
       </c>
       <c r="E83" s="18" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="F83" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="G83" s="20"/>
-      <c r="H83" s="20"/>
-      <c r="I83" s="20"/>
-      <c r="J83" s="20"/>
-      <c r="K83" s="20"/>
-      <c r="L83" s="20"/>
-      <c r="M83" s="20"/>
-      <c r="N83" s="20"/>
-      <c r="O83" s="20"/>
-      <c r="P83" s="20"/>
-      <c r="Q83" s="20"/>
-      <c r="R83" s="20"/>
-      <c r="S83" s="20"/>
-      <c r="T83" s="20"/>
-      <c r="U83" s="20"/>
-      <c r="V83" s="20"/>
-      <c r="W83" s="20"/>
-      <c r="X83" s="20"/>
-      <c r="Y83" s="20"/>
-      <c r="Z83" s="20"/>
-      <c r="AA83" s="20"/>
-      <c r="AB83" s="20"/>
-      <c r="AC83" s="20"/>
-      <c r="AD83" s="20"/>
-      <c r="AE83" s="20"/>
-      <c r="AF83" s="20"/>
+        <v>50</v>
+      </c>
+      <c r="J83" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K83" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L83" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="M83" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="N83" s="18" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="84" spans="1:32">
       <c r="A84" s="17"/>
-      <c r="B84" s="29"/>
-      <c r="C84" s="3"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="3"/>
-      <c r="H84" s="3"/>
-      <c r="J84" s="3"/>
-      <c r="K84" s="3"/>
-      <c r="L84" s="3"/>
-      <c r="M84" s="3"/>
-      <c r="N84" s="3"/>
-      <c r="O84" s="3"/>
-      <c r="P84" s="3"/>
-    </row>
-    <row r="85" spans="1:32">
-      <c r="A85" s="17"/>
-      <c r="B85" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C85" s="18" t="s">
+      <c r="B84" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C84" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="D85" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E85" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="F85" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J85" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K85" s="18" t="s">
+      <c r="D84" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E84" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="F84" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="J84" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K84" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L85" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="M85" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="N85" s="18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="86" spans="1:32">
-      <c r="A86" s="17"/>
-      <c r="B86" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C86" s="18" t="s">
+      <c r="L84" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="M84" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="N84" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="85" spans="1:32" s="34" customFormat="1">
+      <c r="A85" s="35"/>
+      <c r="B85" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="C85" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D86" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E86" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="F86" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J86" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K86" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L86" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="M86" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="N86" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="D85" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="E85" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="F85" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G85" s="35"/>
+      <c r="H85" s="35"/>
+      <c r="I85" s="35"/>
+      <c r="J85" s="35"/>
+      <c r="K85" s="35"/>
+      <c r="L85" s="35"/>
+      <c r="M85" s="35"/>
+      <c r="N85" s="35"/>
+      <c r="O85" s="35"/>
+      <c r="P85" s="35"/>
+      <c r="Q85" s="35"/>
+      <c r="R85" s="35"/>
+      <c r="S85" s="35"/>
+      <c r="T85" s="35"/>
+      <c r="U85" s="35"/>
+      <c r="V85" s="35"/>
+      <c r="W85" s="35"/>
+      <c r="X85" s="35"/>
+      <c r="Y85" s="35"/>
+      <c r="Z85" s="35"/>
+      <c r="AA85" s="35"/>
+      <c r="AB85" s="35"/>
+      <c r="AC85" s="35"/>
+      <c r="AD85" s="35"/>
+      <c r="AE85" s="35"/>
+      <c r="AF85" s="35"/>
+    </row>
+    <row r="86" spans="1:32" s="46" customFormat="1">
+      <c r="A86" s="44"/>
+      <c r="B86" s="45"/>
+      <c r="C86" s="44"/>
+      <c r="D86" s="44"/>
+      <c r="E86" s="44"/>
+      <c r="F86" s="44"/>
+      <c r="G86" s="44"/>
+      <c r="H86" s="44"/>
+      <c r="I86" s="44"/>
+      <c r="J86" s="44"/>
+      <c r="K86" s="44"/>
+      <c r="L86" s="44"/>
+      <c r="M86" s="44"/>
+      <c r="N86" s="44"/>
+      <c r="O86" s="44"/>
+      <c r="P86" s="44"/>
+      <c r="Q86" s="44"/>
+      <c r="R86" s="44"/>
+      <c r="S86" s="44"/>
+      <c r="T86" s="44"/>
+      <c r="U86" s="44"/>
+      <c r="V86" s="44"/>
+      <c r="W86" s="44"/>
+      <c r="X86" s="44"/>
+      <c r="Y86" s="44"/>
+      <c r="Z86" s="44"/>
+      <c r="AA86" s="44"/>
+      <c r="AB86" s="44"/>
+      <c r="AC86" s="44"/>
+      <c r="AD86" s="44"/>
+      <c r="AE86" s="44"/>
+      <c r="AF86" s="44"/>
     </row>
     <row r="87" spans="1:32">
       <c r="A87" s="17"/>
-      <c r="B87" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C87" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D87" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E87" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F87" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J87" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K87" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L87" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="M87" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="N87" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="B87" s="29"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="J87" s="3"/>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+      <c r="M87" s="3"/>
+      <c r="N87" s="3"/>
+      <c r="O87" s="3"/>
+      <c r="P87" s="3"/>
     </row>
     <row r="88" spans="1:32">
       <c r="A88" s="17"/>
@@ -20752,23 +20831,22 @@
         <v>18</v>
       </c>
       <c r="E88" s="18" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="F88" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="H88" s="18"/>
       <c r="J88" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K88" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L88" s="18" t="s">
-        <v>216</v>
+      <c r="L88" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="M88" s="18" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="N88" s="18" t="s">
         <v>50</v>
@@ -20786,23 +20864,22 @@
         <v>18</v>
       </c>
       <c r="E89" s="18" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="F89" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="H89" s="18"/>
       <c r="J89" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K89" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L89" s="18" t="s">
-        <v>216</v>
+      <c r="L89" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="M89" s="18" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="N89" s="18" t="s">
         <v>50</v>
@@ -20820,26 +20897,25 @@
         <v>18</v>
       </c>
       <c r="E90" s="18" t="s">
-        <v>175</v>
+        <v>118</v>
       </c>
       <c r="F90" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H90" s="18"/>
+        <v>50</v>
+      </c>
       <c r="J90" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K90" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L90" s="18" t="s">
-        <v>223</v>
+      <c r="L90" s="32" t="s">
+        <v>216</v>
       </c>
       <c r="M90" s="18" t="s">
-        <v>175</v>
+        <v>118</v>
       </c>
       <c r="N90" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
     </row>
     <row r="91" spans="1:32">
@@ -20854,25 +20930,26 @@
         <v>18</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>193</v>
+        <v>102</v>
       </c>
       <c r="F91" s="18" t="s">
-        <v>130</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="H91" s="18"/>
       <c r="J91" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K91" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L91" s="18" t="s">
-        <v>223</v>
+      <c r="L91" s="32" t="s">
+        <v>216</v>
       </c>
       <c r="M91" s="18" t="s">
-        <v>193</v>
+        <v>102</v>
       </c>
       <c r="N91" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
     </row>
     <row r="92" spans="1:32">
@@ -20887,25 +20964,26 @@
         <v>18</v>
       </c>
       <c r="E92" s="18" t="s">
-        <v>194</v>
+        <v>122</v>
       </c>
       <c r="F92" s="18" t="s">
-        <v>130</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="H92" s="18"/>
       <c r="J92" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K92" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L92" s="18" t="s">
-        <v>223</v>
+      <c r="L92" s="32" t="s">
+        <v>216</v>
       </c>
       <c r="M92" s="18" t="s">
-        <v>194</v>
+        <v>122</v>
       </c>
       <c r="N92" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93" spans="1:32">
@@ -20920,25 +20998,26 @@
         <v>18</v>
       </c>
       <c r="E93" s="18" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="F93" s="18" t="s">
-        <v>50</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="H93" s="18"/>
       <c r="J93" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K93" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L93" s="18" t="s">
+      <c r="L93" s="32" t="s">
         <v>223</v>
       </c>
       <c r="M93" s="18" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="N93" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="94" spans="1:32">
@@ -20953,10 +21032,10 @@
         <v>18</v>
       </c>
       <c r="E94" s="18" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F94" s="18" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="J94" s="17" t="s">
         <v>47</v>
@@ -20964,14 +21043,14 @@
       <c r="K94" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L94" s="18" t="s">
+      <c r="L94" s="32" t="s">
         <v>223</v>
       </c>
       <c r="M94" s="18" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="N94" s="18" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="95" spans="1:32">
@@ -20986,10 +21065,10 @@
         <v>18</v>
       </c>
       <c r="E95" s="18" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="F95" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="J95" s="17" t="s">
         <v>47</v>
@@ -20997,14 +21076,14 @@
       <c r="K95" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L95" s="18" t="s">
+      <c r="L95" s="32" t="s">
         <v>223</v>
       </c>
       <c r="M95" s="18" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="N95" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="96" spans="1:32">
@@ -21019,7 +21098,7 @@
         <v>18</v>
       </c>
       <c r="E96" s="18" t="s">
-        <v>196</v>
+        <v>138</v>
       </c>
       <c r="F96" s="18" t="s">
         <v>50</v>
@@ -21030,11 +21109,11 @@
       <c r="K96" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L96" s="18" t="s">
+      <c r="L96" s="32" t="s">
         <v>223</v>
       </c>
       <c r="M96" s="18" t="s">
-        <v>196</v>
+        <v>138</v>
       </c>
       <c r="N96" s="18" t="s">
         <v>50</v>
@@ -21052,30 +21131,29 @@
         <v>18</v>
       </c>
       <c r="E97" s="18" t="s">
-        <v>119</v>
+        <v>195</v>
       </c>
       <c r="F97" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G97" s="18"/>
       <c r="J97" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K97" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L97" s="18" t="s">
-        <v>216</v>
+      <c r="L97" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="M97" s="18" t="s">
-        <v>119</v>
+        <v>195</v>
       </c>
       <c r="N97" s="18" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="98" spans="1:32">
-      <c r="A98" s="20"/>
+      <c r="A98" s="17"/>
       <c r="B98" s="24" t="s">
         <v>47</v>
       </c>
@@ -21086,50 +21164,29 @@
         <v>18</v>
       </c>
       <c r="E98" s="18" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="F98" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="G98" s="18"/>
-      <c r="H98" s="20"/>
-      <c r="I98" s="20"/>
+        <v>50</v>
+      </c>
       <c r="J98" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K98" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L98" s="18" t="s">
-        <v>216</v>
+      <c r="L98" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="M98" s="18" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="N98" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="O98" s="20"/>
-      <c r="P98" s="20"/>
-      <c r="Q98" s="20"/>
-      <c r="R98" s="20"/>
-      <c r="S98" s="20"/>
-      <c r="T98" s="20"/>
-      <c r="U98" s="20"/>
-      <c r="V98" s="20"/>
-      <c r="W98" s="20"/>
-      <c r="X98" s="20"/>
-      <c r="Y98" s="20"/>
-      <c r="Z98" s="20"/>
-      <c r="AA98" s="20"/>
-      <c r="AB98" s="20"/>
-      <c r="AC98" s="20"/>
-      <c r="AD98" s="20"/>
-      <c r="AE98" s="20"/>
-      <c r="AF98" s="20"/>
+        <v>50</v>
+      </c>
     </row>
     <row r="99" spans="1:32">
-      <c r="A99" s="20"/>
+      <c r="A99" s="17"/>
       <c r="B99" s="24" t="s">
         <v>47</v>
       </c>
@@ -21140,50 +21197,29 @@
         <v>18</v>
       </c>
       <c r="E99" s="18" t="s">
-        <v>134</v>
+        <v>196</v>
       </c>
       <c r="F99" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="G99" s="18"/>
-      <c r="H99" s="20"/>
-      <c r="I99" s="20"/>
+        <v>50</v>
+      </c>
       <c r="J99" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K99" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L99" s="18" t="s">
-        <v>216</v>
+      <c r="L99" s="32" t="s">
+        <v>223</v>
       </c>
       <c r="M99" s="18" t="s">
-        <v>134</v>
+        <v>196</v>
       </c>
       <c r="N99" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="O99" s="20"/>
-      <c r="P99" s="20"/>
-      <c r="Q99" s="20"/>
-      <c r="R99" s="20"/>
-      <c r="S99" s="20"/>
-      <c r="T99" s="20"/>
-      <c r="U99" s="20"/>
-      <c r="V99" s="20"/>
-      <c r="W99" s="20"/>
-      <c r="X99" s="20"/>
-      <c r="Y99" s="20"/>
-      <c r="Z99" s="20"/>
-      <c r="AA99" s="20"/>
-      <c r="AB99" s="20"/>
-      <c r="AC99" s="20"/>
-      <c r="AD99" s="20"/>
-      <c r="AE99" s="20"/>
-      <c r="AF99" s="20"/>
+        <v>50</v>
+      </c>
     </row>
     <row r="100" spans="1:32">
-      <c r="A100" s="20"/>
+      <c r="A100" s="17"/>
       <c r="B100" s="24" t="s">
         <v>47</v>
       </c>
@@ -21194,189 +21230,230 @@
         <v>18</v>
       </c>
       <c r="E100" s="18" t="s">
-        <v>206</v>
+        <v>119</v>
       </c>
       <c r="F100" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G100" s="20"/>
-      <c r="H100" s="20"/>
-      <c r="I100" s="20"/>
-      <c r="J100" s="20"/>
-      <c r="K100" s="20"/>
-      <c r="L100" s="20"/>
-      <c r="M100" s="20"/>
-      <c r="N100" s="20"/>
-      <c r="O100" s="20"/>
-      <c r="P100" s="20"/>
-      <c r="Q100" s="20"/>
-      <c r="R100" s="20"/>
-      <c r="S100" s="20"/>
-      <c r="T100" s="20"/>
-      <c r="U100" s="20"/>
-      <c r="V100" s="20"/>
-      <c r="W100" s="20"/>
-      <c r="X100" s="20"/>
-      <c r="Y100" s="20"/>
-      <c r="Z100" s="20"/>
-      <c r="AA100" s="20"/>
-      <c r="AB100" s="20"/>
-      <c r="AC100" s="20"/>
-      <c r="AD100" s="20"/>
-      <c r="AE100" s="20"/>
-      <c r="AF100" s="20"/>
+      <c r="G100" s="18"/>
+      <c r="J100" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K100" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L100" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="M100" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="N100" s="18" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="101" spans="1:32">
-      <c r="A101" s="17"/>
-      <c r="B101" s="29"/>
-      <c r="C101" s="3"/>
-      <c r="D101" s="3"/>
-      <c r="E101" s="3"/>
-      <c r="F101" s="3"/>
-      <c r="G101" s="3"/>
-      <c r="H101" s="3"/>
-      <c r="J101" s="3"/>
-      <c r="K101" s="3"/>
-      <c r="L101" s="3"/>
-      <c r="M101" s="3"/>
-      <c r="N101" s="3"/>
-      <c r="O101" s="3"/>
-      <c r="P101" s="3"/>
+      <c r="A101" s="20"/>
+      <c r="B101" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D101" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E101" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="F101" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G101" s="18"/>
+      <c r="H101" s="20"/>
+      <c r="I101" s="20"/>
+      <c r="J101" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K101" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L101" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="M101" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="N101" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="O101" s="20"/>
+      <c r="P101" s="20"/>
+      <c r="Q101" s="20"/>
+      <c r="R101" s="20"/>
+      <c r="S101" s="20"/>
+      <c r="T101" s="20"/>
+      <c r="U101" s="20"/>
+      <c r="V101" s="20"/>
+      <c r="W101" s="20"/>
+      <c r="X101" s="20"/>
+      <c r="Y101" s="20"/>
+      <c r="Z101" s="20"/>
+      <c r="AA101" s="20"/>
+      <c r="AB101" s="20"/>
+      <c r="AC101" s="20"/>
+      <c r="AD101" s="20"/>
+      <c r="AE101" s="20"/>
+      <c r="AF101" s="20"/>
     </row>
     <row r="102" spans="1:32">
-      <c r="A102" s="17"/>
-      <c r="B102" s="28" t="s">
+      <c r="A102" s="20"/>
+      <c r="B102" s="24" t="s">
         <v>47</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>255</v>
       </c>
       <c r="D102" s="18" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E102" s="18" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="F102" s="18" t="s">
-        <v>50</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G102" s="18"/>
+      <c r="H102" s="20"/>
+      <c r="I102" s="20"/>
       <c r="J102" s="17" t="s">
         <v>47</v>
       </c>
       <c r="K102" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="L102" s="18" t="s">
-        <v>205</v>
+      <c r="L102" s="32" t="s">
+        <v>216</v>
       </c>
       <c r="M102" s="18" t="s">
-        <v>49</v>
+        <v>134</v>
       </c>
       <c r="N102" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="O102" s="18" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="103" spans="1:32">
-      <c r="A103" s="17"/>
-      <c r="B103" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C103" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="O102" s="20"/>
+      <c r="P102" s="20"/>
+      <c r="Q102" s="20"/>
+      <c r="R102" s="20"/>
+      <c r="S102" s="20"/>
+      <c r="T102" s="20"/>
+      <c r="U102" s="20"/>
+      <c r="V102" s="20"/>
+      <c r="W102" s="20"/>
+      <c r="X102" s="20"/>
+      <c r="Y102" s="20"/>
+      <c r="Z102" s="20"/>
+      <c r="AA102" s="20"/>
+      <c r="AB102" s="20"/>
+      <c r="AC102" s="20"/>
+      <c r="AD102" s="20"/>
+      <c r="AE102" s="20"/>
+      <c r="AF102" s="20"/>
+    </row>
+    <row r="103" spans="1:32" s="34" customFormat="1">
+      <c r="A103" s="35"/>
+      <c r="B103" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="C103" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D103" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E103" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="F103" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J103" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K103" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L103" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="M103" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="N103" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="D103" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E103" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="F103" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G103" s="35"/>
+      <c r="H103" s="35"/>
+      <c r="I103" s="35"/>
+      <c r="J103" s="35"/>
+      <c r="K103" s="35"/>
+      <c r="L103" s="35"/>
+      <c r="M103" s="35"/>
+      <c r="N103" s="35"/>
+      <c r="O103" s="35"/>
+      <c r="P103" s="35"/>
+      <c r="Q103" s="35"/>
+      <c r="R103" s="35"/>
+      <c r="S103" s="35"/>
+      <c r="T103" s="35"/>
+      <c r="U103" s="35"/>
+      <c r="V103" s="35"/>
+      <c r="W103" s="35"/>
+      <c r="X103" s="35"/>
+      <c r="Y103" s="35"/>
+      <c r="Z103" s="35"/>
+      <c r="AA103" s="35"/>
+      <c r="AB103" s="35"/>
+      <c r="AC103" s="35"/>
+      <c r="AD103" s="35"/>
+      <c r="AE103" s="35"/>
+      <c r="AF103" s="35"/>
     </row>
     <row r="104" spans="1:32">
-      <c r="A104" s="17"/>
-      <c r="B104" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C104" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D104" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E104" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="F104" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J104" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K104" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L104" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="M104" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="N104" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="A104" s="20"/>
+      <c r="B104" s="24"/>
+      <c r="C104" s="18"/>
+      <c r="D104" s="18"/>
+      <c r="E104" s="18"/>
+      <c r="F104" s="18"/>
+      <c r="G104" s="20"/>
+      <c r="H104" s="20"/>
+      <c r="I104" s="20"/>
+      <c r="J104" s="20"/>
+      <c r="K104" s="20"/>
+      <c r="L104" s="20"/>
+      <c r="M104" s="20"/>
+      <c r="N104" s="20"/>
+      <c r="O104" s="20"/>
+      <c r="P104" s="20"/>
+      <c r="Q104" s="20"/>
+      <c r="R104" s="20"/>
+      <c r="S104" s="20"/>
+      <c r="T104" s="20"/>
+      <c r="U104" s="20"/>
+      <c r="V104" s="20"/>
+      <c r="W104" s="20"/>
+      <c r="X104" s="20"/>
+      <c r="Y104" s="20"/>
+      <c r="Z104" s="20"/>
+      <c r="AA104" s="20"/>
+      <c r="AB104" s="20"/>
+      <c r="AC104" s="20"/>
+      <c r="AD104" s="20"/>
+      <c r="AE104" s="20"/>
+      <c r="AF104" s="20"/>
     </row>
     <row r="105" spans="1:32">
       <c r="A105" s="17"/>
-      <c r="B105" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C105" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="D105" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E105" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="F105" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="J105" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="K105" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L105" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="M105" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="N105" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="B105" s="29"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3"/>
+      <c r="E105" s="3"/>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+      <c r="J105" s="3"/>
+      <c r="K105" s="3"/>
+      <c r="L105" s="3"/>
+      <c r="M105" s="3"/>
+      <c r="N105" s="3"/>
+      <c r="O105" s="3"/>
+      <c r="P105" s="3"/>
     </row>
     <row r="106" spans="1:32">
       <c r="A106" s="17"/>
@@ -21390,10 +21467,10 @@
         <v>28</v>
       </c>
       <c r="E106" s="18" t="s">
-        <v>175</v>
+        <v>118</v>
       </c>
       <c r="F106" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="J106" s="17" t="s">
         <v>47</v>
@@ -21402,13 +21479,16 @@
         <v>204</v>
       </c>
       <c r="L106" s="18" t="s">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="M106" s="18" t="s">
-        <v>175</v>
+        <v>49</v>
       </c>
       <c r="N106" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
+      </c>
+      <c r="O106" s="18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="107" spans="1:32">
@@ -21423,10 +21503,10 @@
         <v>28</v>
       </c>
       <c r="E107" s="18" t="s">
-        <v>199</v>
+        <v>102</v>
       </c>
       <c r="F107" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="J107" s="17" t="s">
         <v>47</v>
@@ -21435,13 +21515,13 @@
         <v>204</v>
       </c>
       <c r="L107" s="18" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="M107" s="18" t="s">
-        <v>199</v>
+        <v>49</v>
       </c>
       <c r="N107" s="18" t="s">
-        <v>130</v>
+        <v>50</v>
       </c>
     </row>
     <row r="108" spans="1:32">
@@ -21456,10 +21536,10 @@
         <v>28</v>
       </c>
       <c r="E108" s="18" t="s">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="F108" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J108" s="17" t="s">
         <v>47</v>
@@ -21471,10 +21551,10 @@
         <v>224</v>
       </c>
       <c r="M108" s="18" t="s">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="N108" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="109" spans="1:32">
@@ -21489,7 +21569,7 @@
         <v>28</v>
       </c>
       <c r="E109" s="18" t="s">
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="F109" s="18" t="s">
         <v>50</v>
@@ -21501,10 +21581,10 @@
         <v>204</v>
       </c>
       <c r="L109" s="18" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="M109" s="18" t="s">
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="N109" s="18" t="s">
         <v>50</v>
@@ -21522,10 +21602,10 @@
         <v>28</v>
       </c>
       <c r="E110" s="18" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="F110" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="J110" s="17" t="s">
         <v>47</v>
@@ -21537,10 +21617,10 @@
         <v>224</v>
       </c>
       <c r="M110" s="18" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="N110" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="111" spans="1:32">
@@ -21555,10 +21635,10 @@
         <v>28</v>
       </c>
       <c r="E111" s="18" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="F111" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="J111" s="17" t="s">
         <v>47</v>
@@ -21567,13 +21647,13 @@
         <v>204</v>
       </c>
       <c r="L111" s="18" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="M111" s="18" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="N111" s="18" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="112" spans="1:32">
@@ -21588,10 +21668,10 @@
         <v>28</v>
       </c>
       <c r="E112" s="18" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="F112" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="J112" s="17" t="s">
         <v>47</v>
@@ -21600,13 +21680,13 @@
         <v>204</v>
       </c>
       <c r="L112" s="18" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="M112" s="18" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="N112" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -21621,10 +21701,10 @@
         <v>28</v>
       </c>
       <c r="E113" s="18" t="s">
-        <v>161</v>
+        <v>201</v>
       </c>
       <c r="F113" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J113" s="17" t="s">
         <v>47</v>
@@ -21633,13 +21713,13 @@
         <v>204</v>
       </c>
       <c r="L113" s="18" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="M113" s="18" t="s">
-        <v>161</v>
+        <v>201</v>
       </c>
       <c r="N113" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="114" spans="1:14">
@@ -21654,10 +21734,10 @@
         <v>28</v>
       </c>
       <c r="E114" s="18" t="s">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="F114" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J114" s="17" t="s">
         <v>47</v>
@@ -21666,13 +21746,13 @@
         <v>204</v>
       </c>
       <c r="L114" s="18" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="M114" s="18" t="s">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="N114" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115" spans="1:14">
@@ -21687,7 +21767,7 @@
         <v>28</v>
       </c>
       <c r="E115" s="18" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="F115" s="18" t="s">
         <v>50</v>
@@ -21702,7 +21782,7 @@
         <v>218</v>
       </c>
       <c r="M115" s="18" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="N115" s="18" t="s">
         <v>50</v>
@@ -21720,10 +21800,10 @@
         <v>28</v>
       </c>
       <c r="E116" s="18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="F116" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J116" s="17" t="s">
         <v>47</v>
@@ -21735,10 +21815,10 @@
         <v>218</v>
       </c>
       <c r="M116" s="18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="N116" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="117" spans="1:14">
@@ -21753,10 +21833,10 @@
         <v>28</v>
       </c>
       <c r="E117" s="18" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="F117" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J117" s="17" t="s">
         <v>47</v>
@@ -21768,10 +21848,10 @@
         <v>218</v>
       </c>
       <c r="M117" s="18" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="N117" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="118" spans="1:14">
@@ -21786,10 +21866,10 @@
         <v>28</v>
       </c>
       <c r="E118" s="18" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="F118" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J118" s="17" t="s">
         <v>47</v>
@@ -21801,10 +21881,10 @@
         <v>218</v>
       </c>
       <c r="M118" s="18" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="N118" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -21819,10 +21899,10 @@
         <v>28</v>
       </c>
       <c r="E119" s="18" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
       <c r="F119" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="J119" s="17" t="s">
         <v>47</v>
@@ -21834,10 +21914,10 @@
         <v>218</v>
       </c>
       <c r="M119" s="18" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
       <c r="N119" s="18" t="s">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -21852,10 +21932,10 @@
         <v>28</v>
       </c>
       <c r="E120" s="18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F120" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J120" s="17" t="s">
         <v>47</v>
@@ -21867,10 +21947,10 @@
         <v>218</v>
       </c>
       <c r="M120" s="18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="N120" s="18" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="121" spans="1:14">
@@ -21885,10 +21965,10 @@
         <v>28</v>
       </c>
       <c r="E121" s="18" t="s">
-        <v>166</v>
+        <v>129</v>
       </c>
       <c r="F121" s="18" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="J121" s="17" t="s">
         <v>47</v>
@@ -21900,10 +21980,10 @@
         <v>218</v>
       </c>
       <c r="M121" s="18" t="s">
-        <v>166</v>
+        <v>129</v>
       </c>
       <c r="N121" s="18" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
     </row>
     <row r="122" spans="1:14">
@@ -21918,10 +21998,10 @@
         <v>28</v>
       </c>
       <c r="E122" s="18" t="s">
-        <v>91</v>
+        <v>132</v>
       </c>
       <c r="F122" s="18" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="J122" s="17" t="s">
         <v>47</v>
@@ -21933,10 +22013,10 @@
         <v>218</v>
       </c>
       <c r="M122" s="18" t="s">
-        <v>91</v>
+        <v>132</v>
       </c>
       <c r="N122" s="18" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -21951,10 +22031,10 @@
         <v>28</v>
       </c>
       <c r="E123" s="18" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F123" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="J123" s="17" t="s">
         <v>47</v>
@@ -21966,10 +22046,10 @@
         <v>218</v>
       </c>
       <c r="M123" s="18" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="N123" s="18" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -21984,10 +22064,10 @@
         <v>28</v>
       </c>
       <c r="E124" s="18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F124" s="18" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="J124" s="17" t="s">
         <v>47</v>
@@ -21999,10 +22079,10 @@
         <v>218</v>
       </c>
       <c r="M124" s="18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="N124" s="18" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="125" spans="1:14">
@@ -22017,10 +22097,10 @@
         <v>28</v>
       </c>
       <c r="E125" s="18" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F125" s="18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="J125" s="17" t="s">
         <v>47</v>
@@ -22032,10 +22112,10 @@
         <v>218</v>
       </c>
       <c r="M125" s="18" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="N125" s="18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="126" spans="1:14">
@@ -22050,64 +22130,184 @@
         <v>28</v>
       </c>
       <c r="E126" s="18" t="s">
-        <v>206</v>
+        <v>91</v>
       </c>
       <c r="F126" s="18" t="s">
-        <v>120</v>
+        <v>57</v>
+      </c>
+      <c r="J126" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K126" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L126" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M126" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="N126" s="18" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="127" spans="1:14">
       <c r="A127" s="17"/>
+      <c r="B127" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C127" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D127" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E127" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="F127" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J127" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K127" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L127" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M127" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="N127" s="18" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="128" spans="1:14">
       <c r="A128" s="17"/>
-    </row>
-    <row r="129" spans="1:1">
+      <c r="B128" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C128" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D128" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E128" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="F128" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="J128" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K128" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L128" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M128" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="N128" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
       <c r="A129" s="17"/>
-    </row>
-    <row r="130" spans="1:1">
-      <c r="A130" s="17"/>
-    </row>
-    <row r="131" spans="1:1">
+      <c r="B129" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C129" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="D129" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E129" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="F129" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J129" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="K129" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="L129" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M129" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="N129" s="18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14" s="34" customFormat="1">
+      <c r="A130" s="33"/>
+      <c r="B130" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="C130" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="D130" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="E130" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="F130" s="32" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14">
       <c r="A131" s="17"/>
     </row>
-    <row r="132" spans="1:1">
+    <row r="132" spans="1:14">
       <c r="A132" s="17"/>
     </row>
-    <row r="133" spans="1:1">
+    <row r="133" spans="1:14">
       <c r="A133" s="17"/>
     </row>
-    <row r="134" spans="1:1">
+    <row r="134" spans="1:14">
       <c r="A134" s="17"/>
     </row>
-    <row r="135" spans="1:1">
+    <row r="135" spans="1:14">
       <c r="A135" s="17"/>
     </row>
-    <row r="136" spans="1:1">
+    <row r="136" spans="1:14">
       <c r="A136" s="17"/>
     </row>
-    <row r="137" spans="1:1">
+    <row r="137" spans="1:14">
       <c r="A137" s="17"/>
     </row>
-    <row r="138" spans="1:1">
+    <row r="138" spans="1:14">
       <c r="A138" s="17"/>
     </row>
-    <row r="139" spans="1:1">
+    <row r="139" spans="1:14">
       <c r="A139" s="17"/>
     </row>
-    <row r="140" spans="1:1">
+    <row r="140" spans="1:14">
       <c r="A140" s="17"/>
     </row>
-    <row r="141" spans="1:1">
+    <row r="141" spans="1:14">
       <c r="A141" s="17"/>
     </row>
-    <row r="142" spans="1:1">
+    <row r="142" spans="1:14">
       <c r="A142" s="17"/>
     </row>
-    <row r="143" spans="1:1">
+    <row r="143" spans="1:14">
       <c r="A143" s="17"/>
     </row>
-    <row r="144" spans="1:1">
+    <row r="144" spans="1:14">
       <c r="A144" s="17"/>
     </row>
     <row r="145" spans="1:1">
@@ -24485,6 +24685,18 @@
     </row>
     <row r="936" spans="1:1">
       <c r="A936" s="17"/>
+    </row>
+    <row r="937" spans="1:1">
+      <c r="A937" s="17"/>
+    </row>
+    <row r="938" spans="1:1">
+      <c r="A938" s="17"/>
+    </row>
+    <row r="939" spans="1:1">
+      <c r="A939" s="17"/>
+    </row>
+    <row r="940" spans="1:1">
+      <c r="A940" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -24492,6 +24704,7 @@
     <mergeCell ref="J1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -24523,23 +24736,23 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="23"/>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="J1" s="34" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="J1" s="41" t="s">
         <v>260</v>
       </c>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
       <c r="P1" s="13"/>
     </row>
     <row r="2" spans="1:16">
@@ -33804,20 +34017,20 @@
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
-      <c r="I1" s="34" t="s">
+      <c r="I1" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="33" t="s">
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="40"/>
+      <c r="R1" s="40"/>
     </row>
     <row r="2" spans="2:18">
       <c r="B2" s="18" t="s">

</xml_diff>

<commit_message>
erd logical and pysical models finished
</commit_message>
<xml_diff>
--- a/NorthWind WRK.xlsx
+++ b/NorthWind WRK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Analytics_Engineering\analytics-engineering-bootcamp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34157A8-7A24-4FB2-9E2B-E881CCE1078B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85BED856-809E-4314-8693-FBBC0E9C239A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="894" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="894" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BusMatrix-HighLevelEntites-Comp" sheetId="3" r:id="rId1"/>
@@ -64,8 +64,43 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bubi</author>
+  </authors>
+  <commentList>
+    <comment ref="C41" authorId="0" shapeId="0" xr:uid="{B50A1EC3-F611-433C-B381-4C48BA820906}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bubi:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Removed supplier_id
+Added supplier_company</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9440" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9441" uniqueCount="268">
   <si>
     <t>Business Process</t>
   </si>
@@ -868,12 +903,15 @@
   <si>
     <t>source</t>
   </si>
+  <si>
+    <t>updated by transformation tool</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -918,6 +956,19 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="15">
@@ -15802,7 +15853,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <tabColor rgb="FF38761D"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -17918,6 +17969,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -18687,7 +18739,9 @@
         <v>120</v>
       </c>
       <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
+      <c r="H22" s="35" t="s">
+        <v>267</v>
+      </c>
       <c r="I22" s="35"/>
       <c r="J22" s="35"/>
       <c r="K22" s="35"/>

</xml_diff>